<commit_message>
data(na-climate): residual load shape for Power_General, Canada cooling split restored
- TS_POWER_GENERAL: load shape minus the 2025 heating and cooling components per
  NA region (clipped, renormalised); bound to Power_General through new
  Par_TagFuelToTimeseries overlays of the four climate options. Removes the
  double count of heating (v6: winter-peaking in 7 of 9 pools) and cooling (split:
  summer peaks 6-42 % above the 2024 ISO peaks); base-year totals follow the
  measured FEL load shape.
- Canada's cooling back in Power_Buildings_Cooling (COOLING_IN_GENERAL empty).
- builder: build_residual_general, registry rows, check table in derived/.

Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Conversion Script/Set_filter_file_NorthAmerica_climate.xlsx
+++ b/Conversion Script/Set_filter_file_NorthAmerica_climate.xlsx
@@ -2116,7 +2116,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B35"/>
+  <dimension ref="A1:B36"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30.85546875" bestFit="1" customWidth="1" min="1" max="1"/>
@@ -2378,7 +2378,7 @@
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>TS_POWER_BUILDINGS_HEAT_2030</t>
+          <t>TS_POWER_GENERAL</t>
         </is>
       </c>
       <c r="B26" t="n">
@@ -2388,7 +2388,7 @@
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>TS_POWER_BUILDINGS_HEAT_2035</t>
+          <t>TS_POWER_BUILDINGS_HEAT_2030</t>
         </is>
       </c>
       <c r="B27" t="n">
@@ -2398,7 +2398,7 @@
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>TS_POWER_BUILDINGS_COOLING_2030</t>
+          <t>TS_POWER_BUILDINGS_HEAT_2035</t>
         </is>
       </c>
       <c r="B28" t="n">
@@ -2408,7 +2408,7 @@
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>TS_POWER_BUILDINGS_COOLING_2035</t>
+          <t>TS_POWER_BUILDINGS_COOLING_2030</t>
         </is>
       </c>
       <c r="B29" t="n">
@@ -2418,7 +2418,7 @@
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>TS_CF_THERMAL_CCGT</t>
+          <t>TS_POWER_BUILDINGS_COOLING_2035</t>
         </is>
       </c>
       <c r="B30" t="n">
@@ -2428,7 +2428,7 @@
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>TS_CF_THERMAL_OCGT</t>
+          <t>TS_CF_THERMAL_CCGT</t>
         </is>
       </c>
       <c r="B31" t="n">
@@ -2438,7 +2438,7 @@
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>TS_CF_THERMAL_STEAM</t>
+          <t>TS_CF_THERMAL_OCGT</t>
         </is>
       </c>
       <c r="B32" t="n">
@@ -2448,7 +2448,7 @@
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>TS_CF_THERMAL_CCGT_2030</t>
+          <t>TS_CF_THERMAL_STEAM</t>
         </is>
       </c>
       <c r="B33" t="n">
@@ -2458,7 +2458,7 @@
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>TS_CF_THERMAL_OCGT_2030</t>
+          <t>TS_CF_THERMAL_CCGT_2030</t>
         </is>
       </c>
       <c r="B34" t="n">
@@ -2468,10 +2468,20 @@
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
+          <t>TS_CF_THERMAL_OCGT_2030</t>
+        </is>
+      </c>
+      <c r="B35" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
           <t>TS_CF_THERMAL_STEAM_2030</t>
         </is>
       </c>
-      <c r="B35" t="n">
+      <c r="B36" t="n">
         <v>1</v>
       </c>
     </row>

</xml_diff>